<commit_message>
Fix layout overlapping, fix EWS count logic, and set First Shipment date format
</commit_message>
<xml_diff>
--- a/Template_Dashboard_v3.xlsx
+++ b/Template_Dashboard_v3.xlsx
@@ -22,11 +22,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
     <numFmt numFmtId="165" formatCode="#,##0.0;\(#,##0.0\)"/>
     <numFmt numFmtId="166" formatCode="dd\-mmm\-yy"/>
     <numFmt numFmtId="167" formatCode="0.0000"/>
+    <numFmt numFmtId="168" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="61">
     <font>
@@ -874,7 +875,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="216">
+  <cellXfs count="218">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -1400,6 +1401,12 @@
     <xf numFmtId="0" fontId="46" fillId="38" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="60" fillId="39" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="38" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="36" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3992,10 +3999,10 @@
     <mergeCell ref="K33:L33"/>
     <mergeCell ref="B10:F11"/>
     <mergeCell ref="B27:F27"/>
+    <mergeCell ref="G32:J32"/>
     <mergeCell ref="K8:L9"/>
+    <mergeCell ref="P22:Q22"/>
     <mergeCell ref="G15:I15"/>
-    <mergeCell ref="P22:Q22"/>
-    <mergeCell ref="G32:J32"/>
     <mergeCell ref="M21:O21"/>
     <mergeCell ref="G5:L5"/>
     <mergeCell ref="B36:W36"/>
@@ -6394,6 +6401,7 @@
   </sheetData>
   <mergeCells count="63">
     <mergeCell ref="C54:E54"/>
+    <mergeCell ref="C29:E29"/>
     <mergeCell ref="C55:E55"/>
     <mergeCell ref="A15:E15"/>
     <mergeCell ref="C22:E22"/>
@@ -6445,15 +6453,14 @@
     <mergeCell ref="B121:D121"/>
     <mergeCell ref="C33:E33"/>
     <mergeCell ref="B122:D122"/>
-    <mergeCell ref="A40:E40"/>
     <mergeCell ref="C73:E73"/>
     <mergeCell ref="A119:F119"/>
     <mergeCell ref="C64:E64"/>
     <mergeCell ref="C26:E26"/>
-    <mergeCell ref="C29:E29"/>
+    <mergeCell ref="C35:E35"/>
     <mergeCell ref="A58:E58"/>
     <mergeCell ref="C20:E20"/>
-    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="A40:E40"/>
     <mergeCell ref="A87:F87"/>
     <mergeCell ref="C63:E63"/>
   </mergeCells>
@@ -7297,12 +7304,12 @@
           <t>First Shipment</t>
         </is>
       </c>
-      <c r="D67" s="67" t="inlineStr">
+      <c r="D67" s="216" t="inlineStr">
         <is>
           <t>Target (Threshold)</t>
         </is>
       </c>
-      <c r="E67" s="113" t="n">
+      <c r="E67" s="217" t="n">
         <v>46113</v>
       </c>
       <c r="F67" s="114" t="n">
@@ -7372,6 +7379,7 @@
         <v/>
       </c>
     </row>
+    <row r="70"/>
     <row r="71" ht="19.5" customHeight="1" s="132"/>
     <row r="72" ht="15.75" customHeight="1" s="132">
       <c r="C72" s="131" t="inlineStr">

</xml_diff>